<commit_message>
aggregate: raise on same run name, suffix and prefix to generation script
</commit_message>
<xml_diff>
--- a/artifacts/tables/judge-challenge-ranking.xlsx
+++ b/artifacts/tables/judge-challenge-ranking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jn\dev\llm-ensemble\artifacts\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52284B8F-1426-4E2E-8D6E-21A481893986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516C68AB-36B4-47AA-81FB-3839C7746DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E1F2E031-223B-4BB8-9B79-B417D7C8D9D5}"/>
   </bookViews>
@@ -287,19 +287,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Good" xfId="1" builtinId="26"/>
@@ -441,7 +440,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{82DA069E-5747-42BB-8383-ECB6E778D133}" name="Table2" displayName="Table2" ref="C1:E47" totalsRowShown="0" tableBorderDxfId="3">
   <autoFilter ref="C1:E47" xr:uid="{82DA069E-5747-42BB-8383-ECB6E778D133}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:E47">
-    <sortCondition descending="1" ref="E1:E47"/>
+    <sortCondition descending="1" ref="D1:D47"/>
   </sortState>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{2AE2AE10-5299-4DB9-97D3-544CCB58DEE2}" name="submission-id" dataDxfId="2"/>
@@ -784,13 +783,13 @@
         <v>47</v>
       </c>
       <c r="B1"/>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="10" t="s">
+      <c r="E1" s="9" t="s">
         <v>2</v>
       </c>
     </row>
@@ -800,13 +799,13 @@
       </c>
       <c r="B2"/>
       <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" s="4">
-        <v>0.26250000000000001</v>
-      </c>
-      <c r="E2" s="4">
-        <v>0.502</v>
+        <v>42</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.2863</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.49180000000000001</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -815,13 +814,13 @@
       </c>
       <c r="B3"/>
       <c r="C3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0.27739999999999998</v>
-      </c>
-      <c r="E3" s="4">
-        <v>0.49580000000000002</v>
+        <v>28</v>
+      </c>
+      <c r="D3" s="1">
+        <v>0.28170000000000001</v>
+      </c>
+      <c r="E3" s="1">
+        <v>0.48120000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -830,13 +829,13 @@
       </c>
       <c r="B4"/>
       <c r="C4" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0.2863</v>
-      </c>
-      <c r="E4" s="4">
-        <v>0.49180000000000001</v>
+        <v>27</v>
+      </c>
+      <c r="D4" s="1">
+        <v>0.27739999999999998</v>
+      </c>
+      <c r="E4" s="1">
+        <v>0.49580000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -845,13 +844,13 @@
       </c>
       <c r="B5"/>
       <c r="C5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="4">
-        <v>0.2293</v>
-      </c>
-      <c r="E5" s="4">
-        <v>0.48770000000000002</v>
+        <v>44</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.27410000000000001</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.45350000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -860,13 +859,13 @@
       </c>
       <c r="B6"/>
       <c r="C6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="4">
-        <v>0.26540000000000002</v>
-      </c>
-      <c r="E6" s="4">
-        <v>0.48730000000000001</v>
+        <v>43</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0.26879999999999998</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.4556</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -875,13 +874,13 @@
       </c>
       <c r="B7"/>
       <c r="C7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" s="4">
-        <v>0.2271</v>
-      </c>
-      <c r="E7" s="4">
-        <v>0.48699999999999999</v>
+        <v>16</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0.26540000000000002</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0.48730000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -890,13 +889,13 @@
       </c>
       <c r="B8"/>
       <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="4">
-        <v>0.28170000000000001</v>
-      </c>
-      <c r="E8" s="4">
-        <v>0.48120000000000002</v>
+        <v>10</v>
+      </c>
+      <c r="D8" s="1">
+        <v>0.26250000000000001</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0.502</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -904,14 +903,14 @@
         <v>8</v>
       </c>
       <c r="B9"/>
-      <c r="C9" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="7">
-        <v>0.22919999999999999</v>
-      </c>
-      <c r="E9" s="7">
-        <v>0.47520000000000001</v>
+      <c r="C9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0.25890000000000002</v>
+      </c>
+      <c r="E9" s="1">
+        <v>0.38979999999999998</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -922,10 +921,10 @@
       <c r="C10" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="1">
         <v>0.25190000000000001</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E10" s="1">
         <v>0.47010000000000002</v>
       </c>
     </row>
@@ -935,13 +934,13 @@
       </c>
       <c r="B11"/>
       <c r="C11" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="D11" s="4">
-        <v>0.21099999999999999</v>
-      </c>
-      <c r="E11" s="4">
-        <v>0.4642</v>
+        <v>12</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0.2445</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.4551</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -950,13 +949,13 @@
       </c>
       <c r="B12"/>
       <c r="C12" s="1" t="s">
-        <v>43</v>
+        <v>14</v>
       </c>
       <c r="D12" s="4">
-        <v>0.26879999999999998</v>
-      </c>
-      <c r="E12" s="4">
-        <v>0.4556</v>
+        <v>0.23880000000000001</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.4108</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -965,13 +964,13 @@
       </c>
       <c r="B13"/>
       <c r="C13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="4">
-        <v>0.2445</v>
-      </c>
-      <c r="E13" s="4">
-        <v>0.4551</v>
+        <v>38</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0.2293</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.48770000000000002</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -979,14 +978,14 @@
         <v>13</v>
       </c>
       <c r="B14"/>
-      <c r="C14" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="4">
-        <v>0.2064</v>
-      </c>
-      <c r="E14" s="4">
-        <v>0.4536</v>
+      <c r="C14" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="6">
+        <v>0.22919999999999999</v>
+      </c>
+      <c r="E14" s="6">
+        <v>0.47520000000000001</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -995,13 +994,13 @@
       </c>
       <c r="B15"/>
       <c r="C15" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D15" s="4">
-        <v>0.27410000000000001</v>
-      </c>
-      <c r="E15" s="4">
-        <v>0.45350000000000001</v>
+        <v>32</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0.2271</v>
+      </c>
+      <c r="E15" s="1">
+        <v>0.48699999999999999</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -1010,13 +1009,13 @@
       </c>
       <c r="B16"/>
       <c r="C16" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D16" s="4">
-        <v>0.2109</v>
-      </c>
-      <c r="E16" s="4">
-        <v>0.4471</v>
+        <v>35</v>
+      </c>
+      <c r="D16" s="1">
+        <v>0.21099999999999999</v>
+      </c>
+      <c r="E16" s="1">
+        <v>0.4642</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -1025,13 +1024,13 @@
       </c>
       <c r="B17"/>
       <c r="C17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="5">
-        <v>0.23880000000000001</v>
-      </c>
-      <c r="E17" s="4">
-        <v>0.4108</v>
+        <v>13</v>
+      </c>
+      <c r="D17" s="1">
+        <v>0.2109</v>
+      </c>
+      <c r="E17" s="1">
+        <v>0.4471</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -1040,13 +1039,13 @@
       </c>
       <c r="B18"/>
       <c r="C18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="4">
-        <v>0.18229999999999999</v>
-      </c>
-      <c r="E18" s="4">
-        <v>0.40689999999999998</v>
+        <v>26</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0.20880000000000001</v>
+      </c>
+      <c r="E18" s="1">
+        <v>0.3926</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -1054,14 +1053,14 @@
         <v>18</v>
       </c>
       <c r="B19"/>
-      <c r="C19" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="8">
-        <v>0.20610000000000001</v>
-      </c>
-      <c r="E19" s="8">
-        <v>0.39419999999999999</v>
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0.2064</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0.4536</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -1069,14 +1068,14 @@
         <v>19</v>
       </c>
       <c r="B20"/>
-      <c r="C20" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="4">
-        <v>0.20880000000000001</v>
-      </c>
-      <c r="E20" s="4">
-        <v>0.3926</v>
+      <c r="C20" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="D20" s="7">
+        <v>0.20610000000000001</v>
+      </c>
+      <c r="E20" s="7">
+        <v>0.39419999999999999</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -1084,14 +1083,14 @@
         <v>20</v>
       </c>
       <c r="B21"/>
-      <c r="C21" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D21" s="4">
-        <v>0.25890000000000002</v>
-      </c>
-      <c r="E21" s="4">
-        <v>0.38979999999999998</v>
+      <c r="C21" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="D21" s="7">
+        <v>0.2051</v>
+      </c>
+      <c r="E21" s="7">
+        <v>0.38819999999999999</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -1099,14 +1098,14 @@
         <v>21</v>
       </c>
       <c r="B22"/>
-      <c r="C22" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="D22" s="8">
-        <v>0.2051</v>
-      </c>
-      <c r="E22" s="8">
-        <v>0.38819999999999999</v>
+      <c r="C22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="1">
+        <v>0.2006</v>
+      </c>
+      <c r="E22" s="1">
+        <v>0.38729999999999998</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -1115,13 +1114,13 @@
       </c>
       <c r="B23"/>
       <c r="C23" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" s="4">
-        <v>0.18440000000000001</v>
-      </c>
-      <c r="E23" s="4">
-        <v>0.38740000000000002</v>
+        <v>18</v>
+      </c>
+      <c r="D23" s="1">
+        <v>0.1961</v>
+      </c>
+      <c r="E23" s="1">
+        <v>0.38519999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -1130,13 +1129,13 @@
       </c>
       <c r="B24"/>
       <c r="C24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D24" s="4">
-        <v>0.18379999999999999</v>
-      </c>
-      <c r="E24" s="5">
-        <v>0.38740000000000002</v>
+        <v>5</v>
+      </c>
+      <c r="D24" s="1">
+        <v>0.188</v>
+      </c>
+      <c r="E24" s="1">
+        <v>0.3821</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -1145,13 +1144,13 @@
       </c>
       <c r="B25"/>
       <c r="C25" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D25" s="4">
-        <v>0.2006</v>
-      </c>
-      <c r="E25" s="4">
-        <v>0.38729999999999998</v>
+        <v>3</v>
+      </c>
+      <c r="D25" s="1">
+        <v>0.18770000000000001</v>
+      </c>
+      <c r="E25" s="1">
+        <v>0.38190000000000002</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -1160,13 +1159,13 @@
       </c>
       <c r="B26"/>
       <c r="C26" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D26" s="4">
-        <v>0.1845</v>
-      </c>
-      <c r="E26" s="4">
-        <v>0.38719999999999999</v>
+        <v>4</v>
+      </c>
+      <c r="D26" s="1">
+        <v>0.18740000000000001</v>
+      </c>
+      <c r="E26" s="1">
+        <v>0.38119999999999998</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -1175,13 +1174,13 @@
       </c>
       <c r="B27"/>
       <c r="C27" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D27" s="4">
-        <v>0.14710000000000001</v>
-      </c>
-      <c r="E27" s="4">
-        <v>0.38550000000000001</v>
+        <v>7</v>
+      </c>
+      <c r="D27" s="1">
+        <v>0.1845</v>
+      </c>
+      <c r="E27" s="1">
+        <v>0.38719999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -1190,13 +1189,13 @@
       </c>
       <c r="B28"/>
       <c r="C28" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D28" s="4">
-        <v>0.17230000000000001</v>
-      </c>
-      <c r="E28" s="4">
-        <v>0.38529999999999998</v>
+        <v>6</v>
+      </c>
+      <c r="D28" s="1">
+        <v>0.18440000000000001</v>
+      </c>
+      <c r="E28" s="1">
+        <v>0.38740000000000002</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
@@ -1205,13 +1204,13 @@
       </c>
       <c r="B29"/>
       <c r="C29" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D29" s="4">
-        <v>0.1961</v>
+        <v>8</v>
+      </c>
+      <c r="D29" s="1">
+        <v>0.18379999999999999</v>
       </c>
       <c r="E29" s="4">
-        <v>0.38519999999999999</v>
+        <v>0.38740000000000002</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
@@ -1219,14 +1218,14 @@
         <v>29</v>
       </c>
       <c r="B30"/>
-      <c r="C30" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="D30" s="8">
-        <v>0.16450000000000001</v>
-      </c>
-      <c r="E30" s="8">
-        <v>0.38219999999999998</v>
+      <c r="C30" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="1">
+        <v>0.18290000000000001</v>
+      </c>
+      <c r="E30" s="1">
+        <v>0.2888</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
@@ -1235,13 +1234,13 @@
       </c>
       <c r="B31"/>
       <c r="C31" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="4">
-        <v>0.188</v>
-      </c>
-      <c r="E31" s="4">
-        <v>0.3821</v>
+        <v>39</v>
+      </c>
+      <c r="D31" s="1">
+        <v>0.18229999999999999</v>
+      </c>
+      <c r="E31" s="1">
+        <v>0.40689999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
@@ -1250,13 +1249,13 @@
       </c>
       <c r="B32"/>
       <c r="C32" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D32" s="4">
-        <v>0.18770000000000001</v>
-      </c>
-      <c r="E32" s="4">
-        <v>0.38190000000000002</v>
+        <v>40</v>
+      </c>
+      <c r="D32" s="1">
+        <v>0.1757</v>
+      </c>
+      <c r="E32" s="1">
+        <v>0.31440000000000001</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
@@ -1265,13 +1264,13 @@
       </c>
       <c r="B33"/>
       <c r="C33" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D33" s="4">
-        <v>0.18740000000000001</v>
-      </c>
-      <c r="E33" s="4">
-        <v>0.38119999999999998</v>
+        <v>20</v>
+      </c>
+      <c r="D33" s="1">
+        <v>0.17419999999999999</v>
+      </c>
+      <c r="E33" s="1">
+        <v>0.37290000000000001</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
@@ -1280,13 +1279,13 @@
       </c>
       <c r="B34"/>
       <c r="C34" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D34" s="4">
-        <v>0.17419999999999999</v>
-      </c>
-      <c r="E34" s="4">
-        <v>0.37290000000000001</v>
+        <v>21</v>
+      </c>
+      <c r="D34" s="1">
+        <v>0.1741</v>
+      </c>
+      <c r="E34" s="1">
+        <v>0.3579</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
@@ -1295,13 +1294,13 @@
       </c>
       <c r="B35"/>
       <c r="C35" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D35" s="4">
-        <v>0.13270000000000001</v>
-      </c>
-      <c r="E35" s="4">
-        <v>0.36720000000000003</v>
+        <v>37</v>
+      </c>
+      <c r="D35" s="1">
+        <v>0.17230000000000001</v>
+      </c>
+      <c r="E35" s="1">
+        <v>0.38529999999999998</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.35">
@@ -1309,14 +1308,14 @@
         <v>35</v>
       </c>
       <c r="B36"/>
-      <c r="C36" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D36" s="4">
-        <v>0.1741</v>
-      </c>
-      <c r="E36" s="4">
-        <v>0.3579</v>
+      <c r="C36" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D36" s="7">
+        <v>0.16450000000000001</v>
+      </c>
+      <c r="E36" s="7">
+        <v>0.38219999999999998</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -1327,10 +1326,10 @@
       <c r="C37" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D37" s="4">
+      <c r="D37" s="1">
         <v>0.156</v>
       </c>
-      <c r="E37" s="4">
+      <c r="E37" s="1">
         <v>0.32629999999999998</v>
       </c>
     </row>
@@ -1340,13 +1339,13 @@
       </c>
       <c r="B38"/>
       <c r="C38" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D38" s="4">
-        <v>0.12839999999999999</v>
-      </c>
-      <c r="E38" s="4">
-        <v>0.32179999999999997</v>
+        <v>19</v>
+      </c>
+      <c r="D38" s="1">
+        <v>0.14710000000000001</v>
+      </c>
+      <c r="E38" s="1">
+        <v>0.38550000000000001</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
@@ -1355,13 +1354,13 @@
       </c>
       <c r="B39"/>
       <c r="C39" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D39" s="4">
-        <v>0.1236</v>
-      </c>
-      <c r="E39" s="4">
-        <v>0.32069999999999999</v>
+        <v>41</v>
+      </c>
+      <c r="D39" s="1">
+        <v>0.14710000000000001</v>
+      </c>
+      <c r="E39" s="1">
+        <v>0.1623</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
@@ -1370,13 +1369,13 @@
       </c>
       <c r="B40"/>
       <c r="C40" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D40" s="4">
-        <v>0.1137</v>
-      </c>
-      <c r="E40" s="4">
-        <v>0.31480000000000002</v>
+        <v>23</v>
+      </c>
+      <c r="D40" s="1">
+        <v>0.14080000000000001</v>
+      </c>
+      <c r="E40" s="1">
+        <v>0.2712</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
@@ -1385,13 +1384,13 @@
       </c>
       <c r="B41"/>
       <c r="C41" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D41" s="4">
-        <v>0.1757</v>
-      </c>
-      <c r="E41" s="4">
-        <v>0.31440000000000001</v>
+        <v>34</v>
+      </c>
+      <c r="D41" s="1">
+        <v>0.13270000000000001</v>
+      </c>
+      <c r="E41" s="1">
+        <v>0.36720000000000003</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
@@ -1400,13 +1399,13 @@
       </c>
       <c r="B42"/>
       <c r="C42" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D42" s="4">
-        <v>0.18290000000000001</v>
-      </c>
-      <c r="E42" s="4">
-        <v>0.2888</v>
+        <v>30</v>
+      </c>
+      <c r="D42" s="1">
+        <v>0.12839999999999999</v>
+      </c>
+      <c r="E42" s="1">
+        <v>0.32179999999999997</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.35">
@@ -1415,13 +1414,13 @@
       </c>
       <c r="B43"/>
       <c r="C43" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="D43" s="4">
-        <v>7.5399999999999995E-2</v>
-      </c>
-      <c r="E43" s="4">
-        <v>0.28079999999999999</v>
+        <v>36</v>
+      </c>
+      <c r="D43" s="1">
+        <v>0.1236</v>
+      </c>
+      <c r="E43" s="1">
+        <v>0.32069999999999999</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
@@ -1430,13 +1429,13 @@
       </c>
       <c r="B44"/>
       <c r="C44" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D44" s="4">
-        <v>0.14080000000000001</v>
-      </c>
-      <c r="E44" s="4">
-        <v>0.2712</v>
+        <v>24</v>
+      </c>
+      <c r="D44" s="1">
+        <v>0.1137</v>
+      </c>
+      <c r="E44" s="1">
+        <v>0.31480000000000002</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
@@ -1445,13 +1444,13 @@
       </c>
       <c r="B45"/>
       <c r="C45" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D45" s="4">
-        <v>6.0400000000000002E-2</v>
-      </c>
-      <c r="E45" s="4">
-        <v>0.1691</v>
+        <v>25</v>
+      </c>
+      <c r="D45" s="1">
+        <v>7.7899999999999997E-2</v>
+      </c>
+      <c r="E45" s="1">
+        <v>0.1036</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
@@ -1460,13 +1459,13 @@
       </c>
       <c r="B46"/>
       <c r="C46" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D46" s="4">
-        <v>0.14710000000000001</v>
-      </c>
-      <c r="E46" s="4">
-        <v>0.1623</v>
+        <v>33</v>
+      </c>
+      <c r="D46" s="1">
+        <v>7.5399999999999995E-2</v>
+      </c>
+      <c r="E46" s="1">
+        <v>0.28079999999999999</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
@@ -1475,13 +1474,13 @@
       </c>
       <c r="B47"/>
       <c r="C47" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D47" s="4">
-        <v>7.7899999999999997E-2</v>
-      </c>
-      <c r="E47" s="4">
-        <v>0.1036</v>
+        <v>22</v>
+      </c>
+      <c r="D47" s="1">
+        <v>6.0400000000000002E-2</v>
+      </c>
+      <c r="E47" s="1">
+        <v>0.1691</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
table to generate judge challenge ranking
</commit_message>
<xml_diff>
--- a/artifacts/tables/judge-challenge-ranking.xlsx
+++ b/artifacts/tables/judge-challenge-ranking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jn\dev\llm-ensemble\artifacts\tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{516C68AB-36B4-47AA-81FB-3839C7746DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189BDA8F-4AE4-4D4E-A3DA-A74829A8E42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{E1F2E031-223B-4BB8-9B79-B417D7C8D9D5}"/>
   </bookViews>
@@ -173,19 +173,19 @@
     <t>willia-umbrela3</t>
   </si>
   <si>
-    <t>gpt 5.1</t>
-  </si>
-  <si>
-    <t>ensemble(av)</t>
-  </si>
-  <si>
     <t>Rank</t>
   </si>
   <si>
-    <t>ensemble(mvr)</t>
-  </si>
-  <si>
-    <t>ensemble(mva)</t>
+    <t>Ensemble (MVA)</t>
+  </si>
+  <si>
+    <t>Ensemble (MVR)</t>
+  </si>
+  <si>
+    <t>Ensemble (AV)</t>
+  </si>
+  <si>
+    <t>GPT 5.1</t>
   </si>
 </sst>
 </file>
@@ -780,7 +780,7 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B1"/>
       <c r="C1" s="8" t="s">
@@ -979,7 +979,7 @@
       </c>
       <c r="B14"/>
       <c r="C14" s="5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D14" s="6">
         <v>0.22919999999999999</v>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B20"/>
       <c r="C20" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D20" s="7">
         <v>0.20610000000000001</v>
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B21"/>
       <c r="C21" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D21" s="7">
         <v>0.2051</v>
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B36"/>
       <c r="C36" s="7" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D36" s="7">
         <v>0.16450000000000001</v>

</xml_diff>